<commit_message>
docs(v2): regenerate the professor package with Backstage task qualification V2 (HALTED)
A separate BACKSTAGE TASK QUALIFICATION V2 section: summary section 9B, workbook
sheet 22_BACKSTAGE_TASK_QUAL_V2, a README section and an evidence-map entry. The
section states the halt, the runtime-launch defect, the one delivered
observation (not qualification evidence), the identity stopped before delivery,
and that no candidate status was determined; BTQ-T5 remains the only qualified
task. The builder recomputes the two V2 rows from the master run rows and
checks them against the phase's public rows: 146 checks, 0 mismatches; a second
rebuild is byte-identical. The README's workbook-sheet list now also names
sheet 21, which it had omitted.
</commit_message>
<xml_diff>
--- a/study-results/professor-delivery/AFCI_Professor_Results.xlsx
+++ b/study-results/professor-delivery/AFCI_Professor_Results.xlsx
@@ -28,10 +28,11 @@
     <sheet name="19_METRIC_DEFINITIONS" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="20_RECOMPUTATION_AUDIT" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="21_BACKSTAGE_TASK_QUALIFICATION" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="22_BACKSTAGE_TASK_QUAL_V2" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_EXPERIMENT_INVENTORY'!$A$4:$R$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_ALL_RUNS'!$A$4:$AV$166</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_EXPERIMENT_INVENTORY'!$A$4:$R$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_ALL_RUNS'!$A$4:$AV$168</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_FUNCTIONAL_MATRIX'!$A$5:$K$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_ARCHITECTURE_MATRIX'!$A$5:$J$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'06_TOKEN_MATRIX'!$A$5:$M$9</definedName>
@@ -46,10 +47,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'15_EXCLUSIONS'!$A$5:$E$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'16_DECISION_MATRIX'!$A$5:$E$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'17_METRIC_AVAILABILITY'!$A$4:$H$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'18_EVIDENCE_MAP'!$A$4:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'18_EVIDENCE_MAP'!$A$4:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'19_METRIC_DEFINITIONS'!$A$4:$D$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'20_RECOMPUTATION_AUDIT'!$A$10:$D$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'20_RECOMPUTATION_AUDIT'!$A$10:$D$156</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'21_BACKSTAGE_TASK_QUALIFICATION'!$A$6:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'22_BACKSTAGE_TASK_QUAL_V2'!$A$11:$V$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1419,7 +1421,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Compiled 2026-09-25 from study-results/. Reporting only: no benchmark observation was executed and no scientific result was changed. Every figure recomputes from the 162 run/attempt rows; see 20_RECOMPUTATION_AUDIT.</t>
+          <t>Compiled 2026-09-25 from study-results/. Reporting only: no benchmark observation was executed and no scientific result was changed. Every figure recomputes from the 164 run/attempt rows; see 20_RECOMPUTATION_AUDIT.</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1497,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
@@ -1510,7 +1512,7 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
@@ -1525,7 +1527,7 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
@@ -1544,7 +1546,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>15 explicitly invalid; 62 carry no functional verdict at all</t>
+          <t>16 explicitly invalid; 63 carry no functional verdict at all</t>
         </is>
       </c>
     </row>
@@ -1555,11 +1557,11 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>PT08 (3) + PT09 (4, one infrastructure-invalid) + PT10 (3) + Backstage task qualification V1 (16: 15 C1 observations + 1 pre-delivery infrastructure-invalid attempt); instrument evidence, never treatment evidence</t>
+          <t>PT08 (3) + PT09 (4, one infrastructure-invalid) + PT10 (3) + Backstage task qualification V1 (16: 15 C1 observations + 1 pre-delivery infrastructure-invalid attempt) + Backstage task qualification V2 (2, HALTED: 1 observation under a runtime-launch defect + 1 identity stopped before delivery); instrument evidence, never treatment evidence</t>
         </is>
       </c>
     </row>
@@ -1570,11 +1572,11 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>v1 (48), efficiency Attempt 1 (9), diagnostics/qualification (26), Backstage Attempt 1 (7), plus 4 v2 rows. The 12 Backstage Attempt-2 rows outside a functionally valid pair are counted here too, but ONLY the paired EFFICIENCY analysis excludes them: all 18 enter the primary architecture endpoint, which is scored independently of functional validity</t>
+          <t>v1 (48), efficiency Attempt 1 (9), diagnostics/qualification (28), Backstage Attempt 1 (7), plus 4 v2 rows. The 12 Backstage Attempt-2 rows outside a functionally valid pair are counted here too, but ONLY the paired EFFICIENCY analysis excludes them: all 18 enter the primary architecture endpoint, which is scored independently of functional validity</t>
         </is>
       </c>
     </row>
@@ -1630,11 +1632,11 @@
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>12 v1 tasks (T01-T12) + 6 v2 synthetic tasks (PT01, PT04, PT07, PT08, PT09, PT10) + 3 Backstage real-repository tasks (T1, T2, T5) + 5 Backstage qualification candidates (BTQ-T1R, BTQ-T5, BTQ-C02, BTQ-C04, BTQ-C05; C1 only)</t>
+          <t>12 v1 tasks (T01-T12) + 6 v2 synthetic tasks (PT01, PT04, PT07, PT08, PT09, PT10) + 3 Backstage real-repository tasks (T1, T2, T5) + 5 Backstage qualification candidates (BTQ-T1R, BTQ-T5, BTQ-C02, BTQ-C04, BTQ-C05; C1 only) + 2 Backstage V2 candidates that received an attempt before the halt (BTQ2-C01, BTQ2-C02; C1 only)</t>
         </is>
       </c>
     </row>
@@ -7018,7 +7020,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nothing unfavourable is omitted. Of the 162 recorded run/attempt rows, 50 are eligible for any analysis at all, all 50 belong to two non-confirmatory pilots, and 0 are confirmatory.</t>
+          <t>Nothing unfavourable is omitted. Of the 164 recorded run/attempt rows, 50 are eligible for any analysis at all, all 50 belong to two non-confirmatory pilots, and 0 are confirmatory.</t>
         </is>
       </c>
     </row>
@@ -9174,7 +9176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9519,321 +9521,353 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Backstage task qualification V2: HALTED after 1 of 15 - instrument qualification / C1-only / pre-treatment / not AFCI treatment evidence</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>study-results/10_backstage_task_qualification_v2/README.md -&gt; qualification_v2_run_rows.csv (2 rows); docs/v2/AFCI_BACKSTAGE_TASK_QUALIFICATION_V2_HALT_DECISION.md</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>AFCI_MASTER_RUN_RESULTS.csv, experiment_id = V2_BACKSTAGE_TASK_QUALIFICATION_V2 (2 rows)</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>D:\afci-bq2\runs\&lt;run_id&gt;\run_record.json (usage, tools, timing) -&gt; post-hoc hidden scoring, which stops at the private boundary</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>execution plan sha256 2c34bcb8e326a9687b563f0583de5460bb0ce5d6288b9b1f2476422c585bcc55</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>VERIFIED - recomputed from the run rows in 20_RECOMPUTATION_AUDIT; HALTED, no qualification result</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>REPOSITORY AND GOVERNANCE ANCHORS</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
-      <c r="H15" s="4" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
-      <c r="K15" s="4" t="n"/>
-      <c r="L15" s="4" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>what</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>public repo branch</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>study-v2</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>evidence commit (last change to study-results/ outside this package)</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>b98cc65af4c24f110cfa366acca9925fd6f3a202</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  that commit's subject</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>study(backstage): execute task qualification V1 in full and record the result</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>public repo origin</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>https://github.com/thakkarkeyur/afci-bench.git</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>public repo main (v1 base, tag paper-v0)</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>2adc8741acad7ea5423f0bf3d9ad821ff023a35f</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>private evaluator repo HEAD (result provenance only; never pushed)</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>be8374723eaa68c71a81de34946bc1fe8abaa04f</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>governed substrate commit</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>630d3180af0d02a86330dfb599f559e78df65e94</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>governed substrate content hash</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>0198d76c189f38589e872cab4305527c08e86ef736e1550e428e05f9178060f3 (49 entries)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>the MAD - docs/v2/ARCHITECTURE_CONTEXT.md</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>bf6f32b162a23b851596d8b489d938bef10d0b8616a50dcc039873d12ffa7a4d</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>v1 release</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>GitHub ase2026-artifacts-v1 @ 1ba21ad75dacbac5eb87d354a490b088078c30da</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>v1 DOI</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>10.5281/zenodo.19757261</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>TASK BODY HASHES (public)</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="n"/>
-      <c r="J29" s="4" t="n"/>
-      <c r="K29" s="4" t="n"/>
-      <c r="L29" s="4" t="n"/>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="4" t="n"/>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="n"/>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>task</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>used by</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>PT01</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>6c938822fe19cd6e87942a6ee24ec8f604c0883da1b7f80d45216be35d7c9c39</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>efficiency pilot; lower-model pilot</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>PT04</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>f349b150b1d8fe5676fed8460b1840b988ee2bb0a78b1966ef82ae9ce9c8a9b5</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C33" s="9" t="inlineStr">
         <is>
           <t>efficiency pilot; lower-model pilot</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>PT07</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>557caed09420354efbc823c8b72e54b0760ac72847aba0d9c07d99e37ff7d2d7</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>efficiency pilot; lower-model pilot</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>PT08</t>
         </is>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>a31bb515b79cc1e211a662de2a8761c97082dd8bf266ee5b4f660981435badf2</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr">
         <is>
           <t>PT08 diagnostic</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>PT09</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>bac32dc0e7163c9ab1816ac6eea6c98738092cca5cf56715e280f1ec1c0ac44c</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>qualification</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>PT10</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>1b1fe29881b3c9f309939df042272b03164fb3baae878c64345e75edddf36b86</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C37" s="9" t="inlineStr">
         <is>
           <t>qualification</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="22" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
         <is>
           <t>WHAT IS WITHHELD: private opportunity identifiers, rule identifiers, forbidden source and target scopes, anchor paths and hidden acceptance case semantics. They live in the private evaluator repository and the run record refuses to carry them at all. NO NUMERIC RESULT IS WITHHELD.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="22" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>No digest is published in place of a withheld identifier: the public rule catalog and the public corpus together bound the preimage space to a few thousand candidates, so any such digest would be recoverable by enumeration. Traceability instead runs through run ids, task hashes and evaluator manifest digests, which are already public and already high-entropy.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F13"/>
+  <autoFilter ref="A4:F14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10297,7 +10331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11253,120 +11287,209 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>V2_BACKSTAGE_TASK_QUALIFICATION_V2</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Backstage task qualification V2 (instrument qualification, C1-only, pre-treatment; HALTED)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Claude Code CLI 2.1.229 (effort=high, NON_RESET, 96 turns; launched by an extensionless path - see notes)</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>NON_RESET</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>EXECUTION HALTED - RUNTIME LAUNCH DEFECT</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>HALTED - INSTRUMENT QUALIFICATION ONLY (C1-ONLY, PRE-TREATMENT)</t>
+        </is>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>Which V2 candidates reach FUNCTIONAL_VALID &gt;= 2/3 AND TARGET_ARCHITECTURE_VIOLATION &gt;= 1/3 under C1?</t>
+        </is>
+      </c>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>HALTED (SL-V2-BACKSTAGE-TQ-02-H1); no candidate status determined; 0 new QUALIFIED -&gt; INSUFFICIENT ADDITIONAL QUALIFIED TASKS by halt; BTQ-T5 remains the only qualified task</t>
+        </is>
+      </c>
+      <c r="R15" s="8" t="inlineStr">
+        <is>
+          <t>instrument qualification / C1-only / pre-treatment / not AFCI treatment evidence (SL-V2-BACKSTAGE-TQ-02). HALTED after 1 of 15 scheduled observations. The V2 runtime pin launched the frozen 2.1.229 binary by an extensionless path; Claude Code's built-in Grep re-spawns its own executable and could not start (V1, same version as claude.exe: 93 successful Grep/Glob results, 0 such errors). The one delivered observation (Q6, R2) is valid under the frozen classifier (FUNCTIONAL_VALID False, 0/0, 34 turns, 0 files changed, $1.3543) but was produced under the defect and is not used as qualification e</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
           <t>OPEN_SOURCE_COMPLEXITY_STUDY</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Open-source / real-repository complexity study</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>v2 (planned)</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="9" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="M15" s="6" t="inlineStr">
+      <c r="M16" s="9" t="inlineStr">
         <is>
           <t>NOT STARTED</t>
         </is>
       </c>
-      <c r="N15" s="6" t="inlineStr">
+      <c r="N16" s="9" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="O15" s="6" t="inlineStr">
+      <c r="O16" s="9" t="inlineStr">
         <is>
           <t>NOT STARTED</t>
         </is>
       </c>
-      <c r="P15" s="6" t="inlineStr">
+      <c r="P16" s="9" t="inlineStr">
         <is>
           <t>(not yet defined)</t>
         </is>
       </c>
-      <c r="Q15" s="6" t="inlineStr">
+      <c r="Q16" s="9" t="inlineStr">
         <is>
           <t>(none)</t>
         </is>
       </c>
-      <c r="R15" s="8" t="inlineStr">
+      <c r="R16" s="11" t="inlineStr">
         <is>
           <t>Placeholder only. No runs exist. No results are pre-populated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>OPEN_SOURCE_COMPLEXITY_STUDY is a placeholder. No runs exist and no result is pre-populated.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>V2_BACKSTAGE_PILOT_ATTEMPT_2 is COMPLETE: 18 planned, 18 attempted, 18 completed, 18 valid, 0 infrastructure-invalid, 0 retries. It was a WHOLLY NEW execution of the science SL-V2-BACKSTAGE-PILOT-01 froze, with new run ids and new destinations and zero overlap with attempt 1. The frozen 11.1 continuation rule returned NO ARCHITECTURE SIGNAL - DO NOT AUTOMATICALLY EXPAND (criterion 1 PASS, criterion 2 FAIL, criterion 3 PASS). V2_BACKSTAGE_PILOT (attempt 1) stays HALTED and EXCLUDED WHOLESALE and is never pooled with it, replaced by it, or re-run under it.</t>
+          <t>OPEN_SOURCE_COMPLEXITY_STUDY is a placeholder. No runs exist and no result is pre-populated.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
+          <t>V2_BACKSTAGE_PILOT_ATTEMPT_2 is COMPLETE: 18 planned, 18 attempted, 18 completed, 18 valid, 0 infrastructure-invalid, 0 retries. It was a WHOLLY NEW execution of the science SL-V2-BACKSTAGE-PILOT-01 froze, with new run ids and new destinations and zero overlap with attempt 1. The frozen 11.1 continuation rule returned NO ARCHITECTURE SIGNAL - DO NOT AUTOMATICALLY EXPAND (criterion 1 PASS, criterion 2 FAIL, criterion 3 PASS). V2_BACKSTAGE_PILOT (attempt 1) stays HALTED and EXCLUDED WHOLESALE and is never pooled with it, replaced by it, or re-run under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
           <t>V2_BACKSTAGE_TASK_QUALIFICATION_V1 is INSTRUMENT QUALIFICATION / C1-ONLY / PRE-TREATMENT / NOT AFCI TREATMENT EVIDENCE: 15 C1 observations of 5 candidate tasks, 1 of 5 qualified, outcome INSUFFICIENT QUALIFIED TASKS. No C4, no packet, no treatment effect; never pooled with either Backstage attempt. Its 16 rows (15 observations + 1 attempt that failed before task delivery) are all ineligible. See sheet 21.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="22" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>V2_BACKSTAGE_TASK_QUALIFICATION_V2 is HALTED (instrument qualification / C1-only / pre-treatment / not AFCI treatment evidence): 1 of 15 scheduled observations was delivered and it ran under a runtime-launch defect (the built-in Grep tool could not start), so it is not qualification evidence; a second identity was stopped before its task was delivered. No candidate status was determined, 0 tasks newly qualified; BTQ-T5 remains the only qualified task. See sheet 22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>planned / attempted / completed_runs on this sheet are the experiment registry's own counts. V2_EFF_ATTEMPT1's 'completed_runs = 7' is the registry counting its 7 surviving rows; those rows carry run_status = INTACT_GOVERNED_OBSERVATION, not COMPLETE, so a status-based recount of the same rows gives 0. Both readings are correct at their own definition and neither is reconciled away. See sheet 20.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="22" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>Recounted from the run rows, the two analysed pilots agree with the registry exactly: Attempt 2 35 complete / 34 functionally valid / 16 paired blocks, and the lower-model pilot 18 / 17 / 8.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:R15"/>
+  <autoFilter ref="A4:R16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11377,7 +11500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L156"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -11419,7 +11542,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6">
@@ -11429,7 +11552,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7">
@@ -11490,12 +11613,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>164</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>164</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -11637,19 +11760,19 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>task qualification: BTQ-T1R FUNCTIONAL_VALID of 3</t>
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>task qualification V2: master rows (1 delivered observation + 1 stopped before delivery)</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -11659,19 +11782,19 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>task qualification: BTQ-T1R target violations of 3</t>
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>task qualification V2: master rows equal the phase's public rows</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -11683,17 +11806,17 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>task qualification: BTQ-T5 FUNCTIONAL_VALID of 3</t>
+          <t>task qualification V2: rows eligible for any analysis</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -11703,19 +11826,19 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>task qualification: BTQ-T5 target violations of 3</t>
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>task qualification V2: every row carries the instrument-qualification label</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>True</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>True</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -11727,17 +11850,17 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>task qualification: BTQ-C02 FUNCTIONAL_VALID of 3</t>
+          <t>task qualification V2: exactly one task delivered</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -11749,7 +11872,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>task qualification: BTQ-C02 target violations of 3</t>
+          <t>task qualification V2: no row used as qualification evidence</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -11771,17 +11894,17 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>task qualification: BTQ-C04 FUNCTIONAL_VALID of 3</t>
+          <t>task qualification V2: no C4 row</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
@@ -11793,17 +11916,17 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>task qualification: BTQ-C04 target violations of 3</t>
+          <t>task qualification: BTQ-T1R FUNCTIONAL_VALID of 3</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -11815,17 +11938,17 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>task qualification: BTQ-C05 FUNCTIONAL_VALID of 3</t>
+          <t>task qualification: BTQ-T1R target violations of 3</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -11837,17 +11960,17 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>task qualification: BTQ-C05 target violations of 3</t>
+          <t>task qualification: BTQ-T5 FUNCTIONAL_VALID of 3</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -11859,17 +11982,17 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Sonnet blocks observed</t>
+          <t>task qualification: BTQ-T5 target violations of 3</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -11881,17 +12004,17 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Sonnet paired-eligible blocks</t>
+          <t>task qualification: BTQ-C02 FUNCTIONAL_VALID of 3</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -11903,17 +12026,17 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Haiku blocks observed</t>
+          <t>task qualification: BTQ-C02 target violations of 3</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -11925,17 +12048,17 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Haiku paired-eligible blocks</t>
+          <t>task qualification: BTQ-C04 FUNCTIONAL_VALID of 3</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -11947,17 +12070,17 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Sonnet TOTAL_INPUT_TOKENS median C4/C1</t>
+          <t>task qualification: BTQ-C04 target violations of 3</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>1.4014</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>1.4014</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
@@ -11969,17 +12092,17 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Sonnet TOTAL_INPUT_TOKENS paired n</t>
+          <t>task qualification: BTQ-C05 FUNCTIONAL_VALID of 3</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -11991,17 +12114,17 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>Sonnet TOTAL_INPUT_TOKENS C4-lower count</t>
+          <t>task qualification: BTQ-C05 target violations of 3</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
@@ -12013,17 +12136,17 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Sonnet CI_COMMAND_RUNS median C4/C1</t>
+          <t>Sonnet blocks observed</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -12035,7 +12158,7 @@
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Sonnet CI_COMMAND_RUNS paired n</t>
+          <t>Sonnet paired-eligible blocks</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -12057,17 +12180,17 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Sonnet CI_COMMAND_RUNS C4-lower count</t>
+          <t>Haiku blocks observed</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -12079,17 +12202,17 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Sonnet EDIT_AND_WRITE_CALLS median C4/C1</t>
+          <t>Haiku paired-eligible blocks</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>1.9167</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>1.9167</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
@@ -12101,17 +12224,17 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Sonnet EDIT_AND_WRITE_CALLS paired n</t>
+          <t>Sonnet TOTAL_INPUT_TOKENS median C4/C1</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1.4014</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1.4014</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -12123,17 +12246,17 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>Sonnet EDIT_AND_WRITE_CALLS C4-lower count</t>
+          <t>Sonnet TOTAL_INPUT_TOKENS paired n</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
@@ -12145,17 +12268,17 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Sonnet EXPLORATION_CALLS median C4/C1</t>
+          <t>Sonnet TOTAL_INPUT_TOKENS C4-lower count</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>1.3939</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>1.3939</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -12167,17 +12290,17 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>Sonnet EXPLORATION_CALLS paired n</t>
+          <t>Sonnet CI_COMMAND_RUNS median C4/C1</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
@@ -12189,17 +12312,17 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Sonnet EXPLORATION_CALLS C4-lower count</t>
+          <t>Sonnet CI_COMMAND_RUNS paired n</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
@@ -12211,17 +12334,17 @@
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>Sonnet MODEL_WALL_SECONDS median C4/C1</t>
+          <t>Sonnet CI_COMMAND_RUNS C4-lower count</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>1.266</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>1.266</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
@@ -12233,17 +12356,17 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Sonnet MODEL_WALL_SECONDS paired n</t>
+          <t>Sonnet EDIT_AND_WRITE_CALLS median C4/C1</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1.9167</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1.9167</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -12255,17 +12378,17 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>Sonnet MODEL_WALL_SECONDS C4-lower count</t>
+          <t>Sonnet EDIT_AND_WRITE_CALLS paired n</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
@@ -12277,7 +12400,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Sonnet TEST_COMMAND_RUNS paired n</t>
+          <t>Sonnet EDIT_AND_WRITE_CALLS C4-lower count</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
@@ -12299,17 +12422,17 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>Sonnet TOTAL_OUTPUT_TOKENS median C4/C1</t>
+          <t>Sonnet EXPLORATION_CALLS median C4/C1</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>1.4671</t>
+          <t>1.3939</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>1.4671</t>
+          <t>1.3939</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
@@ -12321,17 +12444,17 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Sonnet TOTAL_OUTPUT_TOKENS paired n</t>
+          <t>Sonnet EXPLORATION_CALLS paired n</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -12343,17 +12466,17 @@
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>Sonnet TOTAL_OUTPUT_TOKENS C4-lower count</t>
+          <t>Sonnet EXPLORATION_CALLS C4-lower count</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
@@ -12365,17 +12488,17 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Sonnet TOTAL_TOOL_CALLS median C4/C1</t>
+          <t>Sonnet MODEL_WALL_SECONDS median C4/C1</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>1.1864</t>
+          <t>1.266</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>1.1864</t>
+          <t>1.266</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -12387,7 +12510,7 @@
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>Sonnet TOTAL_TOOL_CALLS paired n</t>
+          <t>Sonnet MODEL_WALL_SECONDS paired n</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
@@ -12409,17 +12532,17 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>Sonnet TOTAL_TOOL_CALLS C4-lower count</t>
+          <t>Sonnet MODEL_WALL_SECONDS C4-lower count</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
@@ -12431,17 +12554,17 @@
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>Sonnet UNIQUE_FILES_READ median C4/C1</t>
+          <t>Sonnet TEST_COMMAND_RUNS paired n</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>1.2111</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>1.2111</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
@@ -12453,17 +12576,17 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>Sonnet UNIQUE_FILES_READ paired n</t>
+          <t>Sonnet TOTAL_OUTPUT_TOKENS median C4/C1</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1.4671</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1.4671</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
@@ -12475,17 +12598,17 @@
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>Sonnet UNIQUE_FILES_READ C4-lower count</t>
+          <t>Sonnet TOTAL_OUTPUT_TOKENS paired n</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
@@ -12497,17 +12620,17 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>Haiku CI_COMMAND_RUNS median C4/C1</t>
+          <t>Sonnet TOTAL_OUTPUT_TOKENS C4-lower count</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
@@ -12519,17 +12642,17 @@
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>Haiku CI_COMMAND_RUNS paired n</t>
+          <t>Sonnet TOTAL_TOOL_CALLS median C4/C1</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.1864</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.1864</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
@@ -12541,17 +12664,17 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>Haiku CI_COMMAND_RUNS C4-lower count</t>
+          <t>Sonnet TOTAL_TOOL_CALLS paired n</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
@@ -12563,17 +12686,17 @@
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>Haiku EDIT_AND_WRITE_CALLS median C4/C1</t>
+          <t>Sonnet TOTAL_TOOL_CALLS C4-lower count</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>1.1741</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>1.1741</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
@@ -12585,17 +12708,17 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>Haiku EDIT_AND_WRITE_CALLS paired n</t>
+          <t>Sonnet UNIQUE_FILES_READ median C4/C1</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.2111</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.2111</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
@@ -12607,17 +12730,17 @@
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>Haiku EDIT_AND_WRITE_CALLS C4-lower count</t>
+          <t>Sonnet UNIQUE_FILES_READ paired n</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
@@ -12629,17 +12752,17 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>Haiku EXPLORATION_CALLS median C4/C1</t>
+          <t>Sonnet UNIQUE_FILES_READ C4-lower count</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>1.7308</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>1.7308</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -12651,17 +12774,17 @@
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>Haiku EXPLORATION_CALLS paired n</t>
+          <t>Haiku CI_COMMAND_RUNS median C4/C1</t>
         </is>
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -12673,17 +12796,17 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>Haiku EXPLORATION_CALLS C4-lower count</t>
+          <t>Haiku CI_COMMAND_RUNS paired n</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -12695,17 +12818,17 @@
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>Haiku MODEL_WALL_SECONDS median C4/C1</t>
+          <t>Haiku CI_COMMAND_RUNS C4-lower count</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>1.5268</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>1.5268</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
@@ -12717,17 +12840,17 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>Haiku MODEL_WALL_SECONDS paired n</t>
+          <t>Haiku EDIT_AND_WRITE_CALLS median C4/C1</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.1741</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.1741</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -12739,17 +12862,17 @@
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>Haiku MODEL_WALL_SECONDS C4-lower count</t>
+          <t>Haiku EDIT_AND_WRITE_CALLS paired n</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -12761,17 +12884,17 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>Haiku TEST_COMMAND_RUNS median C4/C1</t>
+          <t>Haiku EDIT_AND_WRITE_CALLS C4-lower count</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -12783,17 +12906,17 @@
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>Haiku TEST_COMMAND_RUNS paired n</t>
+          <t>Haiku EXPLORATION_CALLS median C4/C1</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.7308</t>
         </is>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.7308</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
@@ -12805,17 +12928,17 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>Haiku TEST_COMMAND_RUNS C4-lower count</t>
+          <t>Haiku EXPLORATION_CALLS paired n</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
@@ -12827,17 +12950,17 @@
     <row r="72">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>Haiku TOTAL_INPUT_TOKENS median C4/C1</t>
+          <t>Haiku EXPLORATION_CALLS C4-lower count</t>
         </is>
       </c>
       <c r="B72" s="9" t="inlineStr">
         <is>
-          <t>2.0372</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>2.0372</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
@@ -12849,17 +12972,17 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>Haiku TOTAL_INPUT_TOKENS paired n</t>
+          <t>Haiku MODEL_WALL_SECONDS median C4/C1</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.5268</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.5268</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -12871,17 +12994,17 @@
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>Haiku TOTAL_INPUT_TOKENS C4-lower count</t>
+          <t>Haiku MODEL_WALL_SECONDS paired n</t>
         </is>
       </c>
       <c r="B74" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
@@ -12893,17 +13016,17 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>Haiku TOTAL_OUTPUT_TOKENS median C4/C1</t>
+          <t>Haiku MODEL_WALL_SECONDS C4-lower count</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>1.7804</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>1.7804</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -12915,17 +13038,17 @@
     <row r="76">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>Haiku TOTAL_OUTPUT_TOKENS paired n</t>
+          <t>Haiku TEST_COMMAND_RUNS median C4/C1</t>
         </is>
       </c>
       <c r="B76" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
@@ -12937,17 +13060,17 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>Haiku TOTAL_OUTPUT_TOKENS C4-lower count</t>
+          <t>Haiku TEST_COMMAND_RUNS paired n</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -12959,17 +13082,17 @@
     <row r="78">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>Haiku TOTAL_TOOL_CALLS median C4/C1</t>
+          <t>Haiku TEST_COMMAND_RUNS C4-lower count</t>
         </is>
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>1.5023</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>1.5023</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
@@ -12981,17 +13104,17 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>Haiku TOTAL_TOOL_CALLS paired n</t>
+          <t>Haiku TOTAL_INPUT_TOKENS median C4/C1</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2.0372</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2.0372</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -13003,17 +13126,17 @@
     <row r="80">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>Haiku TOTAL_TOOL_CALLS C4-lower count</t>
+          <t>Haiku TOTAL_INPUT_TOKENS paired n</t>
         </is>
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
@@ -13025,17 +13148,17 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>Haiku UNIQUE_FILES_READ median C4/C1</t>
+          <t>Haiku TOTAL_INPUT_TOKENS C4-lower count</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -13047,17 +13170,17 @@
     <row r="82">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>Haiku UNIQUE_FILES_READ paired n</t>
+          <t>Haiku TOTAL_OUTPUT_TOKENS median C4/C1</t>
         </is>
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.7804</t>
         </is>
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1.7804</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
@@ -13069,17 +13192,17 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>Haiku UNIQUE_FILES_READ C4-lower count</t>
+          <t>Haiku TOTAL_OUTPUT_TOKENS paired n</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
@@ -13091,17 +13214,17 @@
     <row r="84">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>Sonnet NON_RESET token median (cross-model record)</t>
+          <t>Haiku TOTAL_OUTPUT_TOKENS C4-lower count</t>
         </is>
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
-          <t>1.5582</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>1.5582</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
@@ -13113,17 +13236,17 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>Sonnet NON_RESET token paired n</t>
+          <t>Haiku TOTAL_TOOL_CALLS median C4/C1</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1.5023</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1.5023</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
@@ -13135,17 +13258,17 @@
     <row r="86">
       <c r="A86" s="9" t="inlineStr">
         <is>
-          <t>Sonnet NON_RESET provider-cost median</t>
+          <t>Haiku TOTAL_TOOL_CALLS paired n</t>
         </is>
       </c>
       <c r="B86" s="9" t="inlineStr">
         <is>
-          <t>1.4928</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C86" s="9" t="inlineStr">
         <is>
-          <t>1.4928</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
@@ -13157,17 +13280,17 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>Haiku provider-cost median</t>
+          <t>Haiku TOTAL_TOOL_CALLS C4-lower count</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>1.8865</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>1.8865</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
@@ -13179,17 +13302,17 @@
     <row r="88">
       <c r="A88" s="9" t="inlineStr">
         <is>
-          <t>Sonnet C1 functionally-valid runs</t>
+          <t>Haiku UNIQUE_FILES_READ median C4/C1</t>
         </is>
       </c>
       <c r="B88" s="9" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="C88" s="9" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
@@ -13201,17 +13324,17 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>Sonnet C4 functionally-valid runs</t>
+          <t>Haiku UNIQUE_FILES_READ paired n</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
@@ -13223,17 +13346,17 @@
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
         <is>
-          <t>Haiku C1 functionally-valid runs</t>
+          <t>Haiku UNIQUE_FILES_READ C4-lower count</t>
         </is>
       </c>
       <c r="B90" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
@@ -13245,17 +13368,17 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>Haiku C4 functionally-valid runs</t>
+          <t>Sonnet NON_RESET token median (cross-model record)</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1.5582</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1.5582</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
@@ -13267,7 +13390,7 @@
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
         <is>
-          <t>Haiku C1 applicable opportunities</t>
+          <t>Sonnet NON_RESET token paired n</t>
         </is>
       </c>
       <c r="B92" s="9" t="inlineStr">
@@ -13289,17 +13412,17 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>Haiku C1 violated opportunities</t>
+          <t>Sonnet NON_RESET provider-cost median</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1.4928</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1.4928</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
@@ -13311,17 +13434,17 @@
     <row r="94">
       <c r="A94" s="9" t="inlineStr">
         <is>
-          <t>Haiku C4 applicable opportunities</t>
+          <t>Haiku provider-cost median</t>
         </is>
       </c>
       <c r="B94" s="9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1.8865</t>
         </is>
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1.8865</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
@@ -13333,17 +13456,17 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>Haiku C4 violated opportunities</t>
+          <t>Sonnet C1 functionally-valid runs</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
@@ -13355,17 +13478,17 @@
     <row r="96">
       <c r="A96" s="9" t="inlineStr">
         <is>
-          <t>Haiku captured provider cost, all 18 runs</t>
+          <t>Sonnet C4 functionally-valid runs</t>
         </is>
       </c>
       <c r="B96" s="9" t="inlineStr">
         <is>
-          <t>3.8007</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C96" s="9" t="inlineStr">
         <is>
-          <t>3.8007</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
@@ -13377,17 +13500,17 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>Haiku C1 paired-block cost total</t>
+          <t>Haiku C1 functionally-valid runs</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>1.3862</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
@@ -13399,17 +13522,17 @@
     <row r="98">
       <c r="A98" s="9" t="inlineStr">
         <is>
-          <t>Haiku C4 paired-block cost total</t>
+          <t>Haiku C4 functionally-valid runs</t>
         </is>
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>2.0068</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr">
         <is>
-          <t>2.0068</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
@@ -13419,19 +13542,19 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL_INPUT_TOKENS == input + cache_creation + cache_read on every token-bearing row</t>
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>Haiku C1 applicable opportunities</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
@@ -13443,7 +13566,7 @@
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
         <is>
-          <t>PT08 target-violation runs</t>
+          <t>Haiku C1 violated opportunities</t>
         </is>
       </c>
       <c r="B100" s="9" t="inlineStr">
@@ -13465,17 +13588,17 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>PT09 target-violation runs</t>
+          <t>Haiku C4 applicable opportunities</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
@@ -13487,17 +13610,17 @@
     <row r="102">
       <c r="A102" s="9" t="inlineStr">
         <is>
-          <t>PT10 target-violation runs</t>
+          <t>Haiku C4 violated opportunities</t>
         </is>
       </c>
       <c r="B102" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
@@ -13509,17 +13632,17 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>Haiku paired-block turns_used C1</t>
+          <t>Haiku captured provider cost, all 18 runs</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>3.8007</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>3.8007</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
@@ -13531,17 +13654,17 @@
     <row r="104">
       <c r="A104" s="9" t="inlineStr">
         <is>
-          <t>Haiku paired-block turns_used C4</t>
+          <t>Haiku C1 paired-block cost total</t>
         </is>
       </c>
       <c r="B104" s="9" t="inlineStr">
         <is>
-          <t>309</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="C104" s="9" t="inlineStr">
         <is>
-          <t>309</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
@@ -13553,17 +13676,17 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>Haiku paired-block edit_calls C1</t>
+          <t>Haiku C4 paired-block cost total</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>2.0068</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>2.0068</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
@@ -13573,19 +13696,19 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="9" t="inlineStr">
-        <is>
-          <t>Haiku paired-block edit_calls C4</t>
+      <c r="A106" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL_INPUT_TOKENS == input + cache_creation + cache_read on every token-bearing row</t>
         </is>
       </c>
       <c r="B106" s="9" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C106" s="9" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D106" s="9" t="inlineStr">
@@ -13597,17 +13720,17 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>Haiku paired-block files_reedited C1</t>
+          <t>PT08 target-violation runs</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
@@ -13619,17 +13742,17 @@
     <row r="108">
       <c r="A108" s="9" t="inlineStr">
         <is>
-          <t>Haiku paired-block files_reedited C4</t>
+          <t>PT09 target-violation runs</t>
         </is>
       </c>
       <c r="B108" s="9" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C108" s="9" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
@@ -13641,17 +13764,17 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>Haiku paired-block lines_added C1</t>
+          <t>PT10 target-violation runs</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>1755</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>1755</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
@@ -13663,17 +13786,17 @@
     <row r="110">
       <c r="A110" s="9" t="inlineStr">
         <is>
-          <t>Haiku paired-block lines_added C4</t>
+          <t>Haiku paired-block turns_used C1</t>
         </is>
       </c>
       <c r="B110" s="9" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>229</t>
         </is>
       </c>
       <c r="C110" s="9" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>229</t>
         </is>
       </c>
       <c r="D110" s="9" t="inlineStr">
@@ -13685,17 +13808,17 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>Haiku paired-block lines_removed C1</t>
+          <t>Haiku paired-block turns_used C4</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>309</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>309</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
@@ -13707,17 +13830,17 @@
     <row r="112">
       <c r="A112" s="9" t="inlineStr">
         <is>
-          <t>Haiku paired-block lines_removed C4</t>
+          <t>Haiku paired-block edit_calls C1</t>
         </is>
       </c>
       <c r="B112" s="9" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>54</t>
         </is>
       </c>
       <c r="C112" s="9" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>54</t>
         </is>
       </c>
       <c r="D112" s="9" t="inlineStr">
@@ -13729,17 +13852,17 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>Haiku paired-block net_lines C1</t>
+          <t>Haiku paired-block edit_calls C4</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>1621</t>
+          <t>66</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>1621</t>
+          <t>66</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
@@ -13751,17 +13874,17 @@
     <row r="114">
       <c r="A114" s="9" t="inlineStr">
         <is>
-          <t>Haiku paired-block net_lines C4</t>
+          <t>Haiku paired-block files_reedited C1</t>
         </is>
       </c>
       <c r="B114" s="9" t="inlineStr">
         <is>
-          <t>1746</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C114" s="9" t="inlineStr">
         <is>
-          <t>1746</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D114" s="9" t="inlineStr">
@@ -13773,17 +13896,17 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>Haiku paired-block files_changed C1</t>
+          <t>Haiku paired-block files_reedited C4</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
@@ -13795,17 +13918,17 @@
     <row r="116">
       <c r="A116" s="9" t="inlineStr">
         <is>
-          <t>Haiku paired-block files_changed C4</t>
+          <t>Haiku paired-block lines_added C1</t>
         </is>
       </c>
       <c r="B116" s="9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>1755</t>
         </is>
       </c>
       <c r="C116" s="9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>1755</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr">
@@ -13817,17 +13940,17 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT01 C1</t>
+          <t>Haiku paired-block lines_added C4</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>1.2042</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>1.2042</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
@@ -13839,17 +13962,17 @@
     <row r="118">
       <c r="A118" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT01 C4</t>
+          <t>Haiku paired-block lines_removed C1</t>
         </is>
       </c>
       <c r="B118" s="9" t="inlineStr">
         <is>
-          <t>0.8176</t>
+          <t>134</t>
         </is>
       </c>
       <c r="C118" s="9" t="inlineStr">
         <is>
-          <t>0.8176</t>
+          <t>134</t>
         </is>
       </c>
       <c r="D118" s="9" t="inlineStr">
@@ -13861,17 +13984,17 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT04 C1</t>
+          <t>Haiku paired-block lines_removed C4</t>
         </is>
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>1.0986</t>
+          <t>186</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>1.0986</t>
+          <t>186</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
@@ -13883,17 +14006,17 @@
     <row r="120">
       <c r="A120" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT04 C4</t>
+          <t>Haiku paired-block net_lines C1</t>
         </is>
       </c>
       <c r="B120" s="9" t="inlineStr">
         <is>
-          <t>1.6989</t>
+          <t>1621</t>
         </is>
       </c>
       <c r="C120" s="9" t="inlineStr">
         <is>
-          <t>1.6989</t>
+          <t>1621</t>
         </is>
       </c>
       <c r="D120" s="9" t="inlineStr">
@@ -13905,17 +14028,17 @@
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT07 C1</t>
+          <t>Haiku paired-block net_lines C4</t>
         </is>
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>1.2324</t>
+          <t>1746</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>1.2324</t>
+          <t>1746</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
@@ -13927,17 +14050,17 @@
     <row r="122">
       <c r="A122" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT07 C4</t>
+          <t>Haiku paired-block files_changed C1</t>
         </is>
       </c>
       <c r="B122" s="9" t="inlineStr">
         <is>
-          <t>0.9614</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C122" s="9" t="inlineStr">
         <is>
-          <t>0.9614</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D122" s="9" t="inlineStr">
@@ -13949,17 +14072,17 @@
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT01 C1</t>
+          <t>Haiku paired-block files_changed C4</t>
         </is>
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>1.1603</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>1.1603</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
@@ -13971,17 +14094,17 @@
     <row r="124">
       <c r="A124" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT01 C4</t>
+          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT01 C1</t>
         </is>
       </c>
       <c r="B124" s="9" t="inlineStr">
         <is>
-          <t>1.0137</t>
+          <t>1.2042</t>
         </is>
       </c>
       <c r="C124" s="9" t="inlineStr">
         <is>
-          <t>1.0137</t>
+          <t>1.2042</t>
         </is>
       </c>
       <c r="D124" s="9" t="inlineStr">
@@ -13993,17 +14116,17 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT04 C1</t>
+          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT01 C4</t>
         </is>
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>1.7304</t>
+          <t>0.8176</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>1.7304</t>
+          <t>0.8176</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
@@ -14015,17 +14138,17 @@
     <row r="126">
       <c r="A126" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT04 C4</t>
+          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT04 C1</t>
         </is>
       </c>
       <c r="B126" s="9" t="inlineStr">
         <is>
-          <t>1.4214</t>
+          <t>1.0986</t>
         </is>
       </c>
       <c r="C126" s="9" t="inlineStr">
         <is>
-          <t>1.4214</t>
+          <t>1.0986</t>
         </is>
       </c>
       <c r="D126" s="9" t="inlineStr">
@@ -14037,17 +14160,17 @@
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT07 C1</t>
+          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT04 C4</t>
         </is>
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>1.4085</t>
+          <t>1.6989</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>1.4085</t>
+          <t>1.6989</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
@@ -14059,17 +14182,17 @@
     <row r="128">
       <c r="A128" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT07 C4</t>
+          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT07 C1</t>
         </is>
       </c>
       <c r="B128" s="9" t="inlineStr">
         <is>
-          <t>1.2048</t>
+          <t>1.2324</t>
         </is>
       </c>
       <c r="C128" s="9" t="inlineStr">
         <is>
-          <t>1.2048</t>
+          <t>1.2324</t>
         </is>
       </c>
       <c r="D128" s="9" t="inlineStr">
@@ -14081,17 +14204,17 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead EXPLORATION_CALLS PT01 C1</t>
+          <t>Sonnet reset overhead TOTAL_INPUT_TOKENS PT07 C4</t>
         </is>
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>0.9614</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>0.9614</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
@@ -14103,17 +14226,17 @@
     <row r="130">
       <c r="A130" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead EXPLORATION_CALLS PT01 C4</t>
+          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT01 C1</t>
         </is>
       </c>
       <c r="B130" s="9" t="inlineStr">
         <is>
-          <t>1.3693</t>
+          <t>1.1603</t>
         </is>
       </c>
       <c r="C130" s="9" t="inlineStr">
         <is>
-          <t>1.3693</t>
+          <t>1.1603</t>
         </is>
       </c>
       <c r="D130" s="9" t="inlineStr">
@@ -14125,17 +14248,17 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead EXPLORATION_CALLS PT04 C1</t>
+          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT01 C4</t>
         </is>
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>1.6071</t>
+          <t>1.0137</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>1.6071</t>
+          <t>1.0137</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
@@ -14147,17 +14270,17 @@
     <row r="132">
       <c r="A132" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead EXPLORATION_CALLS PT04 C4</t>
+          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT04 C1</t>
         </is>
       </c>
       <c r="B132" s="9" t="inlineStr">
         <is>
-          <t>1.9091</t>
+          <t>1.7304</t>
         </is>
       </c>
       <c r="C132" s="9" t="inlineStr">
         <is>
-          <t>1.9091</t>
+          <t>1.7304</t>
         </is>
       </c>
       <c r="D132" s="9" t="inlineStr">
@@ -14169,17 +14292,17 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead EXPLORATION_CALLS PT07 C1</t>
+          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT04 C4</t>
         </is>
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>1.8571</t>
+          <t>1.4214</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>1.8571</t>
+          <t>1.4214</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
@@ -14191,17 +14314,17 @@
     <row r="134">
       <c r="A134" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead EXPLORATION_CALLS PT07 C4</t>
+          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT07 C1</t>
         </is>
       </c>
       <c r="B134" s="9" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.4085</t>
         </is>
       </c>
       <c r="C134" s="9" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.4085</t>
         </is>
       </c>
       <c r="D134" s="9" t="inlineStr">
@@ -14213,17 +14336,17 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT01 C1</t>
+          <t>Sonnet reset overhead MODEL_WALL_SECONDS PT07 C4</t>
         </is>
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
-          <t>1.5238</t>
+          <t>1.2048</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>1.5238</t>
+          <t>1.2048</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
@@ -14235,17 +14358,17 @@
     <row r="136">
       <c r="A136" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT01 C4</t>
+          <t>Sonnet reset overhead EXPLORATION_CALLS PT01 C1</t>
         </is>
       </c>
       <c r="B136" s="9" t="inlineStr">
         <is>
-          <t>1.1429</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="C136" s="9" t="inlineStr">
         <is>
-          <t>1.1429</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="D136" s="9" t="inlineStr">
@@ -14257,17 +14380,17 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT04 C1</t>
+          <t>Sonnet reset overhead EXPLORATION_CALLS PT01 C4</t>
         </is>
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>1.357</t>
+          <t>1.3693</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>1.357</t>
+          <t>1.3693</t>
         </is>
       </c>
       <c r="D137" s="6" t="inlineStr">
@@ -14279,17 +14402,17 @@
     <row r="138">
       <c r="A138" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT04 C4</t>
+          <t>Sonnet reset overhead EXPLORATION_CALLS PT04 C1</t>
         </is>
       </c>
       <c r="B138" s="9" t="inlineStr">
         <is>
-          <t>1.8095</t>
+          <t>1.6071</t>
         </is>
       </c>
       <c r="C138" s="9" t="inlineStr">
         <is>
-          <t>1.8095</t>
+          <t>1.6071</t>
         </is>
       </c>
       <c r="D138" s="9" t="inlineStr">
@@ -14301,17 +14424,17 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT07 C1</t>
+          <t>Sonnet reset overhead EXPLORATION_CALLS PT04 C4</t>
         </is>
       </c>
       <c r="B139" s="6" t="inlineStr">
         <is>
-          <t>1.619</t>
+          <t>1.9091</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>1.619</t>
+          <t>1.9091</t>
         </is>
       </c>
       <c r="D139" s="6" t="inlineStr">
@@ -14323,17 +14446,17 @@
     <row r="140">
       <c r="A140" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT07 C4</t>
+          <t>Sonnet reset overhead EXPLORATION_CALLS PT07 C1</t>
         </is>
       </c>
       <c r="B140" s="9" t="inlineStr">
         <is>
-          <t>1.2581</t>
+          <t>1.8571</t>
         </is>
       </c>
       <c r="C140" s="9" t="inlineStr">
         <is>
-          <t>1.2581</t>
+          <t>1.8571</t>
         </is>
       </c>
       <c r="D140" s="9" t="inlineStr">
@@ -14345,17 +14468,17 @@
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset TOKEN overhead lower for C4 in</t>
+          <t>Sonnet reset overhead EXPLORATION_CALLS PT07 C4</t>
         </is>
       </c>
       <c r="B141" s="6" t="inlineStr">
         <is>
-          <t>['PT01', 'PT07']</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>['PT01', 'PT07']</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="D141" s="6" t="inlineStr">
@@ -14367,17 +14490,17 @@
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset WALL overhead lower for C4 in</t>
+          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT01 C1</t>
         </is>
       </c>
       <c r="B142" s="9" t="inlineStr">
         <is>
-          <t>['PT01', 'PT04', 'PT07']</t>
+          <t>1.5238</t>
         </is>
       </c>
       <c r="C142" s="9" t="inlineStr">
         <is>
-          <t>['PT01', 'PT04', 'PT07']</t>
+          <t>1.5238</t>
         </is>
       </c>
       <c r="D142" s="9" t="inlineStr">
@@ -14389,17 +14512,17 @@
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset EXPLORATION overhead lower for C4 in</t>
+          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT01 C4</t>
         </is>
       </c>
       <c r="B143" s="6" t="inlineStr">
         <is>
-          <t>['PT01', 'PT07']</t>
+          <t>1.1429</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
-          <t>['PT01', 'PT07']</t>
+          <t>1.1429</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr">
@@ -14411,17 +14534,17 @@
     <row r="144">
       <c r="A144" s="9" t="inlineStr">
         <is>
-          <t>Sonnet reset TOOL overhead lower for C4 in</t>
+          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT04 C1</t>
         </is>
       </c>
       <c r="B144" s="9" t="inlineStr">
         <is>
-          <t>['PT01', 'PT07']</t>
+          <t>1.357</t>
         </is>
       </c>
       <c r="C144" s="9" t="inlineStr">
         <is>
-          <t>['PT01', 'PT07']</t>
+          <t>1.357</t>
         </is>
       </c>
       <c r="D144" s="9" t="inlineStr">
@@ -14433,17 +14556,17 @@
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>cross-model token difference (frozen record)</t>
+          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT04 C4</t>
         </is>
       </c>
       <c r="B145" s="6" t="inlineStr">
         <is>
-          <t>0.479</t>
+          <t>1.8095</t>
         </is>
       </c>
       <c r="C145" s="6" t="inlineStr">
         <is>
-          <t>0.479</t>
+          <t>1.8095</t>
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr">
@@ -14455,17 +14578,17 @@
     <row r="146">
       <c r="A146" s="9" t="inlineStr">
         <is>
-          <t>exported CSV row count equals the master run rows</t>
+          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT07 C1</t>
         </is>
       </c>
       <c r="B146" s="9" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>1.619</t>
         </is>
       </c>
       <c r="C146" s="9" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>1.619</t>
         </is>
       </c>
       <c r="D146" s="9" t="inlineStr">
@@ -14477,17 +14600,17 @@
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>exported CSV preserves every excluded row</t>
+          <t>Sonnet reset overhead TOTAL_TOOL_CALLS PT07 C4</t>
         </is>
       </c>
       <c r="B147" s="6" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>1.2581</t>
         </is>
       </c>
       <c r="C147" s="6" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>1.2581</t>
         </is>
       </c>
       <c r="D147" s="6" t="inlineStr">
@@ -14499,17 +14622,17 @@
     <row r="148">
       <c r="A148" s="9" t="inlineStr">
         <is>
-          <t>exported CSV carries a reason for every excluded row</t>
+          <t>Sonnet reset TOKEN overhead lower for C4 in</t>
         </is>
       </c>
       <c r="B148" s="9" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>['PT01', 'PT07']</t>
         </is>
       </c>
       <c r="C148" s="9" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>['PT01', 'PT07']</t>
         </is>
       </c>
       <c r="D148" s="9" t="inlineStr">
@@ -14521,17 +14644,17 @@
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>exported CSV introduced no zero where the master had a blank</t>
+          <t>Sonnet reset WALL overhead lower for C4 in</t>
         </is>
       </c>
       <c r="B149" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>['PT01', 'PT04', 'PT07']</t>
         </is>
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>['PT01', 'PT04', 'PT07']</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
@@ -14540,111 +14663,265 @@
         </is>
       </c>
     </row>
-    <row r="151" ht="18" customHeight="1">
-      <c r="A151" s="3" t="inlineStr">
-        <is>
-          <t>SCOPE NOTES - where a figure elsewhere in the evidence package is stated at a different scope</t>
-        </is>
-      </c>
-      <c r="B151" s="4" t="n"/>
-      <c r="C151" s="4" t="n"/>
-      <c r="D151" s="4" t="n"/>
-      <c r="E151" s="4" t="n"/>
-      <c r="F151" s="4" t="n"/>
-      <c r="G151" s="4" t="n"/>
-      <c r="H151" s="4" t="n"/>
-      <c r="I151" s="4" t="n"/>
-      <c r="J151" s="4" t="n"/>
-      <c r="K151" s="4" t="n"/>
-      <c r="L151" s="4" t="n"/>
-    </row>
-    <row r="152" ht="30" customHeight="1">
-      <c r="A152" s="5" t="inlineStr">
-        <is>
-          <t>figure</t>
-        </is>
-      </c>
-      <c r="B152" s="5" t="inlineStr">
-        <is>
-          <t>this package reports</t>
-        </is>
-      </c>
-      <c r="C152" s="5" t="inlineStr">
-        <is>
-          <t>note</t>
+    <row r="150">
+      <c r="A150" s="9" t="inlineStr">
+        <is>
+          <t>Sonnet reset EXPLORATION overhead lower for C4 in</t>
+        </is>
+      </c>
+      <c r="B150" s="9" t="inlineStr">
+        <is>
+          <t>['PT01', 'PT07']</t>
+        </is>
+      </c>
+      <c r="C150" s="9" t="inlineStr">
+        <is>
+          <t>['PT01', 'PT07']</t>
+        </is>
+      </c>
+      <c r="D150" s="9" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet reset TOOL overhead lower for C4 in</t>
+        </is>
+      </c>
+      <c r="B151" s="6" t="inlineStr">
+        <is>
+          <t>['PT01', 'PT07']</t>
+        </is>
+      </c>
+      <c r="C151" s="6" t="inlineStr">
+        <is>
+          <t>['PT01', 'PT07']</t>
+        </is>
+      </c>
+      <c r="D151" s="6" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="9" t="inlineStr">
+        <is>
+          <t>cross-model token difference (frozen record)</t>
+        </is>
+      </c>
+      <c r="B152" s="9" t="inlineStr">
+        <is>
+          <t>0.479</t>
+        </is>
+      </c>
+      <c r="C152" s="9" t="inlineStr">
+        <is>
+          <t>0.479</t>
+        </is>
+      </c>
+      <c r="D152" s="9" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>Haiku CI command runs, C1 vs C4</t>
-        </is>
-      </c>
-      <c r="B153" s="8" t="inlineStr">
-        <is>
-          <t>over the 8 PAIRED BLOCKS: C1 13, C4 8. Over ALL 9 runs per arm: C1 15, C4 9. Both scopes are stated, and neither is mixed.</t>
-        </is>
-      </c>
-      <c r="C153" s="8" t="inlineStr">
-        <is>
-          <t>AFCI_RESULTS_SUMMARY.md reports 'C4 needed fewer failed CI cycles (9 vs 13)'. Two things differ here. First, the lower-model evidence carries a CI COMMAND COUNT, not a failed-cycle count, so this package reports it as a command count; the Sonnet pilot does record a genuine FAILED_TEST_OR_CI_CYCLES figure (C1 2, C4 1 over 16 blocks) and that is reported as one. Second, '9 vs 13' takes its two numbers from different scopes: 9 is C4 over all 9 runs and 13 is C1 over the 8 paired blocks. Held to one scope the pair is 8 vs 13 (paired) or 9 vs 15 (all runs). The direction is the same either way; the magnitude is not.</t>
+          <t>exported CSV row count equals the master run rows</t>
+        </is>
+      </c>
+      <c r="B153" s="6" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
+      </c>
+      <c r="C153" s="6" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
+      </c>
+      <c r="D153" s="6" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="9" t="inlineStr">
         <is>
-          <t>Haiku 'files changed', C1 25 vs C4 30</t>
-        </is>
-      </c>
-      <c r="B154" s="11" t="inlineStr">
-        <is>
-          <t>reported as FILES_CHANGED (worktree diff), and UNIQUE_FILES_MODIFIED (tool-call count) is reported beside it as a separate metric: C1 27, C4 30</t>
-        </is>
-      </c>
-      <c r="C154" s="11" t="inlineStr">
-        <is>
-          <t>The two disagree on PT07/C1/R2 (6 files written, 4 files different). Merging them would misreport one of the two.</t>
+          <t>exported CSV preserves every excluded row</t>
+        </is>
+      </c>
+      <c r="B154" s="9" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="C154" s="9" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="6" t="inlineStr">
         <is>
-          <t>Sonnet reset-overhead scope</t>
+          <t>exported CSV carries a reason for every excluded row</t>
         </is>
       </c>
       <c r="B155" s="6" t="inlineStr">
         <is>
-          <t>16 of 18 repetition pairs</t>
-        </is>
-      </c>
-      <c r="C155" s="8" t="inlineStr">
-        <is>
-          <t>A repetition contributes only when BOTH of its runs are functionally valid, which drops PT01/C4/R1 and PT04/C1/R1. Including them changes PT04's C1 overhead, so the scope is stated rather than assumed.</t>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="C155" s="6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D155" s="6" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="9" t="inlineStr">
         <is>
+          <t>exported CSV introduced no zero where the master had a blank</t>
+        </is>
+      </c>
+      <c r="B156" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C156" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D156" s="9" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="18" customHeight="1">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>SCOPE NOTES - where a figure elsewhere in the evidence package is stated at a different scope</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="n"/>
+      <c r="C158" s="4" t="n"/>
+      <c r="D158" s="4" t="n"/>
+      <c r="E158" s="4" t="n"/>
+      <c r="F158" s="4" t="n"/>
+      <c r="G158" s="4" t="n"/>
+      <c r="H158" s="4" t="n"/>
+      <c r="I158" s="4" t="n"/>
+      <c r="J158" s="4" t="n"/>
+      <c r="K158" s="4" t="n"/>
+      <c r="L158" s="4" t="n"/>
+    </row>
+    <row r="159" ht="30" customHeight="1">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>figure</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>this package reports</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="6" t="inlineStr">
+        <is>
+          <t>Haiku CI command runs, C1 vs C4</t>
+        </is>
+      </c>
+      <c r="B160" s="8" t="inlineStr">
+        <is>
+          <t>over the 8 PAIRED BLOCKS: C1 13, C4 8. Over ALL 9 runs per arm: C1 15, C4 9. Both scopes are stated, and neither is mixed.</t>
+        </is>
+      </c>
+      <c r="C160" s="8" t="inlineStr">
+        <is>
+          <t>AFCI_RESULTS_SUMMARY.md reports 'C4 needed fewer failed CI cycles (9 vs 13)'. Two things differ here. First, the lower-model evidence carries a CI COMMAND COUNT, not a failed-cycle count, so this package reports it as a command count; the Sonnet pilot does record a genuine FAILED_TEST_OR_CI_CYCLES figure (C1 2, C4 1 over 16 blocks) and that is reported as one. Second, '9 vs 13' takes its two numbers from different scopes: 9 is C4 over all 9 runs and 13 is C1 over the 8 paired blocks. Held to one scope the pair is 8 vs 13 (paired) or 9 vs 15 (all runs). The direction is the same either way; the magnitude is not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="9" t="inlineStr">
+        <is>
+          <t>Haiku 'files changed', C1 25 vs C4 30</t>
+        </is>
+      </c>
+      <c r="B161" s="11" t="inlineStr">
+        <is>
+          <t>reported as FILES_CHANGED (worktree diff), and UNIQUE_FILES_MODIFIED (tool-call count) is reported beside it as a separate metric: C1 27, C4 30</t>
+        </is>
+      </c>
+      <c r="C161" s="11" t="inlineStr">
+        <is>
+          <t>The two disagree on PT07/C1/R2 (6 files written, 4 files different). Merging them would misreport one of the two.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet reset-overhead scope</t>
+        </is>
+      </c>
+      <c r="B162" s="6" t="inlineStr">
+        <is>
+          <t>16 of 18 repetition pairs</t>
+        </is>
+      </c>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>A repetition contributes only when BOTH of its runs are functionally valid, which drops PT01/C4/R1 and PT04/C1/R1. Including them changes PT04's C1 overhead, so the scope is stated rather than assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="9" t="inlineStr">
+        <is>
           <t>Sonnet block count</t>
         </is>
       </c>
-      <c r="B156" s="9" t="inlineStr">
+      <c r="B163" s="9" t="inlineStr">
         <is>
           <t>19 observed blocks against 18 scheduled</t>
         </is>
       </c>
-      <c r="C156" s="11" t="inlineStr">
+      <c r="C163" s="11" t="inlineStr">
         <is>
           <t>The refused record (sequence 12) carries no reset state, so it forms its own block key. The frozen analysis sees the same 19. The row is preserved exactly as recorded and is not repaired.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A10:D149"/>
+  <autoFilter ref="A10:D156"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16658,13 +16935,437 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="70" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BACKSTAGE TASK QUALIFICATION V2 - HALTED - instrument qualification / C1-only / pre-treatment / not AFCI treatment evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SL-V2-BACKSTAGE-TQ-02 (pre-registered), halted by SL-V2-BACKSTAGE-TQ-02-H1 after 1 of 15 scheduled observations. C1 only: no C4 observation, no architecture packet, no treatment effect. Never pooled with Backstage Attempts 1/2 or Task Qualification V1, which are unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>EVERY ROW ON THIS SHEET IS: INSTRUMENT QUALIFICATION / C1-ONLY / PRE-TREATMENT / NOT AFCI TREATMENT EVIDENCE. NONE IS A QUALIFICATION RESULT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>OUTCOME - HALTED; NO CANDIDATE STATUS DETERMINED; 0 NEW QUALIFIED</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>WHAT HAPPENED: the V2 runtime pin launched the frozen Claude Code 2.1.229 binary by an extensionless path. Version and digest checks passed, but the built-in Grep tool re-spawns its own executable, which Windows cannot resolve without an executable extension, so the tool could not start. Task Qualification V1 ran the same version under its usual executable name and never hit this (93 successful Grep/Glob results, 0 such errors). No pre-data gate exercised a built-in tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>The one delivered observation is valid under the frozen classifier but was produced under the defect and is NOT used as qualification evidence. The executor was stopped before the second task was delivered (no model process, $0). Offered a fix under a recorded deviation, continuing unchanged or stopping, the Study Lead stopped the phase. Frozen selection rule, first branch: fewer than two newly QUALIFIED = INSUFFICIENT ADDITIONAL QUALIFIED TASKS - reached by halt, not by measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>All five V2 candidates remain statically qualified instruments (reference matrix, visible gate, task/oracle alignment, leakage audit and real preparation all green before data); any future use needs a new pre-data decision. Qualified inventory for a future study: BTQ-T5 (V1) only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>SELECTION LIMITATION (recorded before data): qualification selects tasks with measurable baseline architecture pressure; a study built on it estimates AFCI behaviour on ARCHITECTURE-PRESSURE-QUALIFIED BACKSTAGE TASKS only, never an unbiased estimate over arbitrary Backstage changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>EVERY ATTEMPT - instrument qualification / C1-only / pre-treatment / not AFCI treatment evidence</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>sequence</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>task_id</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>repetition</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>execution_attempt</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>disposition</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>task_delivered</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>observation_valid</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>functional_valid</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>semantic_passed</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>semantic_total</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>architecture_applicable_opportunities</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>architecture_violated_opportunities</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>target_violation</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>turns_used</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>permission_denials</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>files_changed</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>cost_usd</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>runtime_launch_defect</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>used_as_qualification_evidence</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>labels</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>BTQ2-C01</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>afci-bq2-btq2-c01-c1-real-r2-non-reset-a1-f961c268b634</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>SCIENTIFIC_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="P12" s="6" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S12" s="6" t="inlineStr">
+        <is>
+          <t>1.3543155</t>
+        </is>
+      </c>
+      <c r="T12" s="6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="U12" s="6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="V12" s="8" t="inlineStr">
+        <is>
+          <t>instrument qualification; C1-only; pre-treatment; not AFCI treatment evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>BTQ2-C02</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>afci-bq2-btq2-c02-c1-real-r3-non-reset-a1-44ed8f6fddca</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>STOPPED_BEFORE_DELIVERY</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr"/>
+      <c r="K13" s="9" t="inlineStr"/>
+      <c r="L13" s="9" t="inlineStr"/>
+      <c r="M13" s="9" t="inlineStr"/>
+      <c r="N13" s="9" t="inlineStr"/>
+      <c r="O13" s="9" t="inlineStr"/>
+      <c r="P13" s="9" t="inlineStr"/>
+      <c r="Q13" s="9" t="inlineStr"/>
+      <c r="R13" s="9" t="inlineStr"/>
+      <c r="S13" s="9" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="T13" s="9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="U13" s="9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="V13" s="11" t="inlineStr">
+        <is>
+          <t>instrument qualification; C1-only; pre-treatment; not AFCI treatment evidence</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A11:V13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV166"/>
+  <dimension ref="A1:AV168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16720,7 +17421,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>All 162 run / attempt records</t>
+          <t>All 164 run / attempt records</t>
         </is>
       </c>
     </row>
@@ -40187,8 +40888,298 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
+        <is>
+          <t>V2_BACKSTAGE_TASK_QUALIFICATION_V2</t>
+        </is>
+      </c>
+      <c r="B167" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C167" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" s="6" t="inlineStr">
+        <is>
+          <t>afci-bq2-btq2-c01-c1-real-r2-non-reset-a1-f961c268b634</t>
+        </is>
+      </c>
+      <c r="E167" s="6" t="inlineStr">
+        <is>
+          <t>BTQ2-C01</t>
+        </is>
+      </c>
+      <c r="F167" s="6" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="G167" s="6" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H167" s="6" t="inlineStr">
+        <is>
+          <t>NON_RESET</t>
+        </is>
+      </c>
+      <c r="I167" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J167" s="6" t="inlineStr">
+        <is>
+          <t>BACKSTAGE_TASK_QUALIFICATION_V2_C1_ONLY</t>
+        </is>
+      </c>
+      <c r="K167" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="L167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M167" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="N167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P167" s="6" t="n"/>
+      <c r="Q167" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="R167" s="7" t="n">
+        <v>90280</v>
+      </c>
+      <c r="S167" s="7" t="n">
+        <v>1903015</v>
+      </c>
+      <c r="T167" s="7" t="n">
+        <v>1993362</v>
+      </c>
+      <c r="U167" s="7" t="n">
+        <v>16102</v>
+      </c>
+      <c r="V167" s="23" t="n">
+        <v>222.261</v>
+      </c>
+      <c r="W167" s="23" t="n">
+        <v>1475.084</v>
+      </c>
+      <c r="X167" s="19" t="n">
+        <v>1.3543155</v>
+      </c>
+      <c r="Y167" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="Z167" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="AA167" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="AB167" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD167" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="AE167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG167" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="AH167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN167" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO167" s="6" t="inlineStr">
+        <is>
+          <t>NOT_APPLICABLE_NON_RESET</t>
+        </is>
+      </c>
+      <c r="AP167" s="6" t="inlineStr">
+        <is>
+          <t>UNDER_CEILING</t>
+        </is>
+      </c>
+      <c r="AQ167" s="6" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="AR167" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AS167" s="8" t="inlineStr">
+        <is>
+          <t>instrument qualification / C1-only / pre-treatment / not AFCI treatment evidence (SL-V2-BACKSTAGE-TQ-02); produced under the V2 runtime-launch defect (the built-in Grep tool could not start) and not used as qualification evidence; phase HALTED (SL-V2-BACKSTAGE-TQ-02-H1)</t>
+        </is>
+      </c>
+      <c r="AT167" s="8" t="inlineStr">
+        <is>
+          <t>D:\afci-bq2\runs\afci-bq2-btq2-c01-c1-real-r2-non-reset-a1-f961c268b634</t>
+        </is>
+      </c>
+      <c r="AU167" s="8" t="inlineStr">
+        <is>
+          <t>task_sha256=3b91a6ae7be948a2ab26bd2035abd18e1c0853981c888f1928ed0f05aff7cdf0</t>
+        </is>
+      </c>
+      <c r="AV167" s="8" t="inlineStr">
+        <is>
+          <t>slot=Q6; rule_family=family E: extension contract placement / ownership; model_invoked=True; model_readback=claude-sonnet-5; effort_readback=VALIDATED; runtime=2.1.229; turns_used=34/96; completion=COMPLETED_NATURALLY; permission_denials=4; gate_command_runs=0; files_changed=0; target_violation=False; labels=instrument qualification; C1-only; pre-treatment; not AFCI treatment evidence; runtime_launch_defect=grep_tool_could_not_start; used_as_qualification_evidence=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="9" t="inlineStr">
+        <is>
+          <t>V2_BACKSTAGE_TASK_QUALIFICATION_V2</t>
+        </is>
+      </c>
+      <c r="B168" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C168" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D168" s="9" t="inlineStr">
+        <is>
+          <t>afci-bq2-btq2-c02-c1-real-r3-non-reset-a1-44ed8f6fddca</t>
+        </is>
+      </c>
+      <c r="E168" s="9" t="inlineStr">
+        <is>
+          <t>BTQ2-C02</t>
+        </is>
+      </c>
+      <c r="F168" s="9" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="G168" s="9" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H168" s="9" t="inlineStr">
+        <is>
+          <t>NON_RESET</t>
+        </is>
+      </c>
+      <c r="I168" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J168" s="9" t="inlineStr">
+        <is>
+          <t>BACKSTAGE_TASK_QUALIFICATION_V2_C1_ONLY</t>
+        </is>
+      </c>
+      <c r="K168" s="9" t="n"/>
+      <c r="L168" s="9" t="n"/>
+      <c r="M168" s="9" t="n"/>
+      <c r="N168" s="9" t="n"/>
+      <c r="O168" s="9" t="n"/>
+      <c r="P168" s="9" t="n"/>
+      <c r="Q168" s="9" t="n"/>
+      <c r="R168" s="9" t="n"/>
+      <c r="S168" s="9" t="n"/>
+      <c r="T168" s="9" t="n"/>
+      <c r="U168" s="9" t="n"/>
+      <c r="V168" s="9" t="n"/>
+      <c r="W168" s="9" t="n"/>
+      <c r="X168" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y168" s="9" t="n"/>
+      <c r="Z168" s="9" t="n"/>
+      <c r="AA168" s="9" t="n"/>
+      <c r="AB168" s="9" t="n"/>
+      <c r="AC168" s="9" t="n"/>
+      <c r="AD168" s="9" t="n"/>
+      <c r="AE168" s="9" t="n"/>
+      <c r="AF168" s="9" t="n"/>
+      <c r="AG168" s="9" t="n"/>
+      <c r="AH168" s="9" t="n"/>
+      <c r="AI168" s="9" t="n"/>
+      <c r="AJ168" s="9" t="n"/>
+      <c r="AK168" s="9" t="n"/>
+      <c r="AL168" s="9" t="n"/>
+      <c r="AM168" s="9" t="n"/>
+      <c r="AN168" s="9" t="n"/>
+      <c r="AO168" s="9" t="inlineStr">
+        <is>
+          <t>NOT_APPLICABLE_NON_RESET</t>
+        </is>
+      </c>
+      <c r="AP168" s="9" t="n"/>
+      <c r="AQ168" s="9" t="inlineStr">
+        <is>
+          <t>STOPPED_BEFORE_DELIVERY_NON_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AR168" s="9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AS168" s="11" t="inlineStr">
+        <is>
+          <t>instrument qualification / C1-only / pre-treatment / not AFCI treatment evidence (SL-V2-BACKSTAGE-TQ-02); stopped by the operator during workspace preparation, before task delivery, on discovering the runtime-launch defect; no model process; phase HALTED (SL-V2-BACKSTAGE-TQ-02-H1)</t>
+        </is>
+      </c>
+      <c r="AT168" s="11" t="inlineStr">
+        <is>
+          <t>D:\afci-bq2\runs\afci-bq2-btq2-c02-c1-real-r3-non-reset-a1-44ed8f6fddca</t>
+        </is>
+      </c>
+      <c r="AU168" s="11" t="inlineStr">
+        <is>
+          <t>task_sha256=79252b843f675948a98b5f41a5d06b9775a4ffa5abd3dfe7fde8259ee6968aa0</t>
+        </is>
+      </c>
+      <c r="AV168" s="11" t="inlineStr">
+        <is>
+          <t>slot=Q7; model_invoked=False; task_delivered=False; no execution_attempt=2 activated</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:AV166"/>
+  <autoFilter ref="A4:AV168"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -42613,7 +43604,7 @@
     <row r="29">
       <c r="A29" s="22" t="inlineStr">
         <is>
-          <t>Programme-wide: 93 of 162 run rows carry input-token evidence and 77 carry output-token evidence. v1 (48 rows), Attempt 1 (9 rows) and the PT08/PT09/PT10 diagnostics (10 rows) predate or do not use the token instrumentation, and their cells are blank rather than 0. The one Backstage task-qualification attempt that failed before its task was delivered invoked no model, so it has no token record either.</t>
+          <t>Programme-wide: 94 of 164 run rows carry input-token evidence and 78 carry output-token evidence. v1 (48 rows), Attempt 1 (9 rows) and the PT08/PT09/PT10 diagnostics (10 rows) predate or do not use the token instrumentation, and their cells are blank rather than 0. The one Backstage task-qualification attempt that failed before its task was delivered, and the V2 identity stopped before delivery, invoked no model, so they have no token record either.</t>
         </is>
       </c>
     </row>
@@ -43134,10 +44125,10 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C23" s="29" t="n">
-        <v>91.8297894</v>
+        <v>93.18410489999999</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
@@ -43176,7 +44167,7 @@
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>CAVEAT: this is captured cost, not total study cost. 84 of 162 run rows carry no provider-cost record at all - all 48 v1 rows (v1 predates cost instrumentation), all 9 Attempt-1 rows, all 10 diagnostic/qualification rows, 16 of 17 Sonnet RESET rows, and the one refused run. Money was spent on those runs; the runtime simply never reported it in a form the record could carry. Do not read the total as what the programme cost.</t>
+          <t>CAVEAT: this is captured cost, not total study cost. 84 of 164 run rows carry no provider-cost record at all - all 48 v1 rows (v1 predates cost instrumentation), all 9 Attempt-1 rows, all 10 diagnostic/qualification rows, 16 of 17 Sonnet RESET rows, and the one refused run. Money was spent on those runs; the runtime simply never reported it in a form the record could carry. Do not read the total as what the programme cost.</t>
         </is>
       </c>
     </row>

</xml_diff>